<commit_message>
Safe Direct Write Excel for QC-17 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-17.xlsx
+++ b/FM-MN-07_QC-17.xlsx
@@ -1751,7 +1751,11 @@
       </c>
       <c r="J6" s="26" t="n"/>
       <c r="K6" s="26" t="n"/>
-      <c r="L6" s="26" t="n"/>
+      <c r="L6" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="26" t="n"/>
       <c r="N6" s="26" t="n"/>
       <c r="O6" s="26" t="n"/>
@@ -1796,7 +1800,11 @@
       </c>
       <c r="J7" s="26" t="n"/>
       <c r="K7" s="26" t="n"/>
-      <c r="L7" s="26" t="n"/>
+      <c r="L7" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="26" t="n"/>
       <c r="N7" s="26" t="n"/>
       <c r="O7" s="26" t="n"/>
@@ -1841,7 +1849,11 @@
       </c>
       <c r="J8" s="26" t="n"/>
       <c r="K8" s="26" t="n"/>
-      <c r="L8" s="26" t="n"/>
+      <c r="L8" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="26" t="n"/>
       <c r="N8" s="26" t="n"/>
       <c r="O8" s="26" t="n"/>
@@ -1886,7 +1898,11 @@
       </c>
       <c r="J9" s="26" t="n"/>
       <c r="K9" s="26" t="n"/>
-      <c r="L9" s="26" t="n"/>
+      <c r="L9" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="26" t="n"/>
       <c r="N9" s="26" t="n"/>
       <c r="O9" s="26" t="n"/>
@@ -1931,7 +1947,11 @@
       </c>
       <c r="J10" s="26" t="n"/>
       <c r="K10" s="26" t="n"/>
-      <c r="L10" s="26" t="n"/>
+      <c r="L10" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="26" t="n"/>
       <c r="N10" s="26" t="n"/>
       <c r="O10" s="26" t="n"/>
@@ -1970,7 +1990,11 @@
       </c>
       <c r="J11" s="38" t="n"/>
       <c r="K11" s="38" t="n"/>
-      <c r="L11" s="38" t="n"/>
+      <c r="L11" s="39" t="inlineStr">
+        <is>
+          <t>เชาวรินทร์</t>
+        </is>
+      </c>
       <c r="M11" s="38" t="n"/>
       <c r="N11" s="38" t="n"/>
       <c r="O11" s="38" t="n"/>
@@ -2148,8 +2172,8 @@
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
+    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="P11:P12"/>
-    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="AG11:AG12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>

</xml_diff>